<commit_message>
Updated Excel to have Business Unit Field
</commit_message>
<xml_diff>
--- a/Example - Time Tracking Excel.xlsx
+++ b/Example - Time Tracking Excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sentineltech365-my.sharepoint.com/personal/jlake_sentinel_com/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sentineltech365-my.sharepoint.com/personal/jlake_sentinel_com/Documents/Documents/Coding/TimeEntry-Tampermonkey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1103" documentId="8_{33648ED4-A4DB-41CF-8BC5-CC71B52D30A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82DF08CE-8DDC-4687-A5DA-7C95BFB4F538}"/>
+  <xr:revisionPtr revIDLastSave="1108" documentId="8_{33648ED4-A4DB-41CF-8BC5-CC71B52D30A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87D3C416-55B0-4553-BCD9-99AAA5E69768}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA0B4115-3D2D-4F3B-BCF9-11BB5874BF0E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BA0B4115-3D2D-4F3B-BCF9-11BB5874BF0E}"/>
   </bookViews>
   <sheets>
     <sheet name="Time Tracking" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="253">
   <si>
     <t>Date</t>
   </si>
@@ -814,6 +814,12 @@
   </si>
   <si>
     <t>cr Holdings Inc</t>
+  </si>
+  <si>
+    <t>Business Unit</t>
+  </si>
+  <si>
+    <t>Enterprise Applications</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1252,8 @@
     <col min="6" max="7" width="34.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="26" width="9.140625" style="5"/>
   </cols>
   <sheetData>
@@ -1281,6 +1288,9 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" t="s">
+        <v>251</v>
+      </c>
       <c r="L1" t="s">
         <v>10</v>
       </c>
@@ -1320,6 +1330,9 @@
       <c r="J2" t="s">
         <v>17</v>
       </c>
+      <c r="K2" t="s">
+        <v>252</v>
+      </c>
       <c r="M2" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M2:N2" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Floracraft-Azure Landing Zone</v>
@@ -1360,6 +1373,9 @@
       <c r="J3" t="s">
         <v>17</v>
       </c>
+      <c r="K3" t="s">
+        <v>252</v>
+      </c>
       <c r="M3" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M3:N3" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -1400,6 +1416,9 @@
       <c r="J4" t="s">
         <v>17</v>
       </c>
+      <c r="K4" t="s">
+        <v>252</v>
+      </c>
       <c r="M4" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M4" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>QCR Holdings-Azure Event Hub</v>
@@ -1436,6 +1455,9 @@
       <c r="J5" t="s">
         <v>17</v>
       </c>
+      <c r="K5" t="s">
+        <v>252</v>
+      </c>
       <c r="M5" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M5:N5" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Floracraft-Azure Landing Zone</v>
@@ -1476,6 +1498,9 @@
       <c r="J6" t="s">
         <v>17</v>
       </c>
+      <c r="K6" t="s">
+        <v>252</v>
+      </c>
       <c r="M6" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M6:N6" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Floracraft-Azure Landing Zone</v>
@@ -1516,6 +1541,9 @@
       <c r="J7" t="s">
         <v>17</v>
       </c>
+      <c r="K7" t="s">
+        <v>252</v>
+      </c>
       <c r="M7" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M7" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Aurorium-Azure Services</v>
@@ -1552,6 +1580,9 @@
       <c r="J8" t="s">
         <v>17</v>
       </c>
+      <c r="K8" t="s">
+        <v>252</v>
+      </c>
       <c r="M8" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M8:N8" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Floracraft-Azure Landing Zone</v>
@@ -1592,6 +1623,9 @@
       <c r="J9" t="s">
         <v>17</v>
       </c>
+      <c r="K9" t="s">
+        <v>252</v>
+      </c>
       <c r="M9" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M9" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Clark County Library District-Azure Accelerate Assessment</v>
@@ -1628,6 +1662,9 @@
       <c r="J10" t="s">
         <v>17</v>
       </c>
+      <c r="K10" t="s">
+        <v>252</v>
+      </c>
       <c r="M10" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M10:N10" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -1668,6 +1705,9 @@
       <c r="J11" t="s">
         <v>17</v>
       </c>
+      <c r="K11" t="s">
+        <v>252</v>
+      </c>
       <c r="M11" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M11" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>National Council of State Boards of Nursing-Microsoft Resource</v>
@@ -1704,6 +1744,9 @@
       <c r="J12" t="s">
         <v>17</v>
       </c>
+      <c r="K12" t="s">
+        <v>252</v>
+      </c>
       <c r="M12" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M12" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>L.E.K Consulting-Azure Networking Assessment</v>
@@ -1740,6 +1783,9 @@
       <c r="J13" t="s">
         <v>17</v>
       </c>
+      <c r="K13" t="s">
+        <v>252</v>
+      </c>
       <c r="M13" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M13" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>WK Kellogg-AVD and Windows 365</v>
@@ -1776,6 +1822,9 @@
       <c r="J14" t="s">
         <v>17</v>
       </c>
+      <c r="K14" t="s">
+        <v>252</v>
+      </c>
       <c r="M14" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M14" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>L.E.K Consulting-Azure Networking Assessment</v>
@@ -1809,6 +1858,9 @@
       <c r="J15" t="s">
         <v>17</v>
       </c>
+      <c r="K15" t="s">
+        <v>252</v>
+      </c>
       <c r="M15" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M15" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>National Council of State Boards of Nursing-Microsoft Resource</v>
@@ -1845,6 +1897,9 @@
       <c r="J16" t="s">
         <v>17</v>
       </c>
+      <c r="K16" t="s">
+        <v>252</v>
+      </c>
       <c r="M16" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M16" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Aurorium-Azure Services</v>
@@ -1881,6 +1936,9 @@
       <c r="J17" t="s">
         <v>17</v>
       </c>
+      <c r="K17" t="s">
+        <v>252</v>
+      </c>
       <c r="M17" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M17:N17" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -1921,6 +1979,9 @@
       <c r="J18" t="s">
         <v>17</v>
       </c>
+      <c r="K18" t="s">
+        <v>252</v>
+      </c>
       <c r="M18" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M18:N18" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -1961,6 +2022,9 @@
       <c r="J19" t="s">
         <v>17</v>
       </c>
+      <c r="K19" t="s">
+        <v>252</v>
+      </c>
       <c r="M19" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M19" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>City of Des Plaines-Azure Domain Controller Migration</v>
@@ -1997,6 +2061,9 @@
       <c r="J20" t="s">
         <v>17</v>
       </c>
+      <c r="K20" t="s">
+        <v>252</v>
+      </c>
       <c r="M20" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M20:N20" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -2037,6 +2104,9 @@
       <c r="J21" t="s">
         <v>17</v>
       </c>
+      <c r="K21" t="s">
+        <v>252</v>
+      </c>
       <c r="M21" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M21" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>WK Kellogg-AVD and Windows 365</v>
@@ -2073,6 +2143,9 @@
       <c r="J22" t="s">
         <v>17</v>
       </c>
+      <c r="K22" t="s">
+        <v>252</v>
+      </c>
       <c r="M22" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M22:N22" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -2113,6 +2186,9 @@
       <c r="J23" t="s">
         <v>17</v>
       </c>
+      <c r="K23" t="s">
+        <v>252</v>
+      </c>
       <c r="M23" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M23" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>WK Kellogg-AVD and Windows 365</v>
@@ -2149,6 +2225,9 @@
       <c r="J24" t="s">
         <v>17</v>
       </c>
+      <c r="K24" t="s">
+        <v>252</v>
+      </c>
       <c r="M24" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M24:N24" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -2189,6 +2268,9 @@
       <c r="J25" t="s">
         <v>17</v>
       </c>
+      <c r="K25" t="s">
+        <v>252</v>
+      </c>
       <c r="M25" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M25:N25" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Brightstar Care-Azure Network Services</v>
@@ -2229,6 +2311,9 @@
       <c r="J26" t="s">
         <v>17</v>
       </c>
+      <c r="K26" t="s">
+        <v>252</v>
+      </c>
       <c r="M26" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M26:N26" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -2269,6 +2354,9 @@
       <c r="J27" t="s">
         <v>17</v>
       </c>
+      <c r="K27" t="s">
+        <v>252</v>
+      </c>
       <c r="M27" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M27" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Sylvan-AVD Proof of Concept</v>
@@ -2305,6 +2393,9 @@
       <c r="J28" t="s">
         <v>17</v>
       </c>
+      <c r="K28" t="s">
+        <v>252</v>
+      </c>
       <c r="M28" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M28:N28" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Floracraft-Azure Landing Zone</v>
@@ -2345,6 +2436,9 @@
       <c r="J29" t="s">
         <v>17</v>
       </c>
+      <c r="K29" t="s">
+        <v>252</v>
+      </c>
       <c r="M29" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M29" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Atlas Healthcare Partners-Windows 365 Jumpstart</v>
@@ -2381,6 +2475,9 @@
       <c r="J30" t="s">
         <v>17</v>
       </c>
+      <c r="K30" t="s">
+        <v>252</v>
+      </c>
       <c r="M30" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M30" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Aurorium-Azure Services</v>
@@ -2417,6 +2514,9 @@
       <c r="J31" t="s">
         <v>17</v>
       </c>
+      <c r="K31" t="s">
+        <v>252</v>
+      </c>
       <c r="M31" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M31:N31" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -2457,6 +2557,9 @@
       <c r="J32" t="s">
         <v>17</v>
       </c>
+      <c r="K32" t="s">
+        <v>252</v>
+      </c>
       <c r="M32" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M32" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>QCR Holdings-Azure Event Hub</v>
@@ -2493,6 +2596,9 @@
       <c r="J33" t="s">
         <v>17</v>
       </c>
+      <c r="K33" t="s">
+        <v>252</v>
+      </c>
       <c r="M33" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M33" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Aurorium-Azure Services</v>
@@ -2529,6 +2635,9 @@
       <c r="J34" t="s">
         <v>17</v>
       </c>
+      <c r="K34" t="s">
+        <v>252</v>
+      </c>
       <c r="M34" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M34" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Atlas Healthcare Partners-Windows 365 Jumpstart</v>
@@ -2565,6 +2674,9 @@
       <c r="J35" t="s">
         <v>17</v>
       </c>
+      <c r="K35" t="s">
+        <v>252</v>
+      </c>
       <c r="M35" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M35:N35" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -2605,6 +2717,9 @@
       <c r="J36" t="s">
         <v>17</v>
       </c>
+      <c r="K36" t="s">
+        <v>252</v>
+      </c>
       <c r="M36" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M36" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Atlas Healthcare Partners-Windows 365 Jumpstart</v>
@@ -2641,6 +2756,9 @@
       <c r="J37" t="s">
         <v>17</v>
       </c>
+      <c r="K37" t="s">
+        <v>252</v>
+      </c>
       <c r="M37" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M37" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>L.E.K Consulting-Azure Networking Assessment</v>
@@ -2677,6 +2795,9 @@
       <c r="J38" t="s">
         <v>17</v>
       </c>
+      <c r="K38" t="s">
+        <v>252</v>
+      </c>
       <c r="M38" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M38" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Atlas Healthcare Partners-Windows 365 Jumpstart</v>
@@ -2713,6 +2834,9 @@
       <c r="J39" t="s">
         <v>17</v>
       </c>
+      <c r="K39" t="s">
+        <v>252</v>
+      </c>
       <c r="M39" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M39:N39" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -2753,6 +2877,9 @@
       <c r="J40" t="s">
         <v>17</v>
       </c>
+      <c r="K40" t="s">
+        <v>252</v>
+      </c>
       <c r="M40" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M40:N40" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>SPAR Group-Server Project Design</v>
@@ -2793,6 +2920,9 @@
       <c r="J41" t="s">
         <v>17</v>
       </c>
+      <c r="K41" t="s">
+        <v>252</v>
+      </c>
       <c r="M41" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M41" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>QCR Holdings-Azure Event Hub</v>
@@ -2829,6 +2959,9 @@
       <c r="J42" t="s">
         <v>17</v>
       </c>
+      <c r="K42" t="s">
+        <v>252</v>
+      </c>
       <c r="M42" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M42" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Aurorium-Azure Services</v>
@@ -2865,6 +2998,9 @@
       <c r="J43" t="s">
         <v>17</v>
       </c>
+      <c r="K43" t="s">
+        <v>252</v>
+      </c>
       <c r="M43" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M43:N43" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Bradford Exchange Ltd-Azure Land Zone-Discovery_Workshops_Documentation</v>
@@ -2905,6 +3041,9 @@
       <c r="J44" t="s">
         <v>17</v>
       </c>
+      <c r="K44" t="s">
+        <v>252</v>
+      </c>
       <c r="M44" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M44:N44" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -2945,6 +3084,9 @@
       <c r="J45" t="s">
         <v>17</v>
       </c>
+      <c r="K45" t="s">
+        <v>252</v>
+      </c>
       <c r="M45" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M45" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>National Council of State Boards of Nursing-Microsoft Resource</v>
@@ -2981,6 +3123,9 @@
       <c r="J46" t="s">
         <v>17</v>
       </c>
+      <c r="K46" t="s">
+        <v>252</v>
+      </c>
       <c r="M46" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M46:N46" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>Credit Interlink-Production to Azure Migration T_M</v>
@@ -3021,6 +3166,9 @@
       <c r="J47" t="s">
         <v>17</v>
       </c>
+      <c r="K47" t="s">
+        <v>252</v>
+      </c>
       <c r="M47" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M47" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>City of Des Plaines-Azure Domain Controller Migration</v>
@@ -3051,6 +3199,9 @@
       <c r="J48" t="s">
         <v>17</v>
       </c>
+      <c r="K48" t="s">
+        <v>252</v>
+      </c>
       <c r="M48" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="M48" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>
         <v>#VALUE!</v>
@@ -3086,6 +3237,9 @@
       </c>
       <c r="J49" t="s">
         <v>17</v>
+      </c>
+      <c r="K49" t="s">
+        <v>252</v>
       </c>
       <c r="M49" s="5" t="str" cm="1">
         <f t="array" aca="1" ref="M49" ca="1">_xlfn.TEXTSPLIT(_xlfn.TEXTJOIN(",",TRUE,_xlfn._xlws.FILTER('Active Projects'!B:B, 'Active Projects'!A:A=INDIRECT("B"&amp;ROW()))),",")</f>

</xml_diff>